<commit_message>
Data: update group stage quiniela predictions to include draws for close matches
</commit_message>
<xml_diff>
--- a/Mundial 2026 (fase de grupos).xlsx
+++ b/Mundial 2026 (fase de grupos).xlsx
@@ -529,7 +529,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -551,7 +551,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">

</xml_diff>

<commit_message>
Feat: precargar resultados del 13-14 de junio y actualizar Excel
</commit_message>
<xml_diff>
--- a/Mundial 2026 (fase de grupos).xlsx
+++ b/Mundial 2026 (fase de grupos).xlsx
@@ -643,7 +643,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">

</xml_diff>

<commit_message>
Feat: precargar resultados de Espana vs Cabo Verde, Belgica vs Egipto, Arabia vs Uruguay
</commit_message>
<xml_diff>
--- a/Mundial 2026 (fase de grupos).xlsx
+++ b/Mundial 2026 (fase de grupos).xlsx
@@ -728,7 +728,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">

</xml_diff>